<commit_message>
Adding in release files for Back Exp Board
</commit_message>
<xml_diff>
--- a/Back_Expansion/Back_Expansion_Base/Release/PCBA/02.BOM/Bill_Of_Materials-BoM(Main).xlsx
+++ b/Back_Expansion/Back_Expansion_Base/Release/PCBA/02.BOM/Bill_Of_Materials-BoM(Main).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JK\Desktop\src_moddo\moddoMOUSE-PCB\Back_Expansion\Back_Expansion_Base\Release\PCBA\02.BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ED1C8397-374F-4B59-83D5-BAD01AD39BED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{535D988F-6731-46FE-BBAE-E9DE68840809}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9984" yWindow="-17388" windowWidth="41496" windowHeight="16776" xr2:uid="{88662ADC-41FE-4431-8F68-8BF36DF6F1F4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="61656" windowHeight="16776" xr2:uid="{180905D2-C27F-4D47-A6CB-DA5C3BB1CCA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill_Of_Materials-BoM(Main)" sheetId="1" r:id="rId1"/>
@@ -821,7 +821,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB95387B-B144-41AC-83E1-733AA2828CCC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66025895-7BB7-480D-A0AD-4DE637999D73}">
   <dimension ref="A1:J22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>